<commit_message>
long overdue update on all scripts
</commit_message>
<xml_diff>
--- a/analysis/results_semen_china.xlsx
+++ b/analysis/results_semen_china.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AK2"/>
+  <dimension ref="A1:AB2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -452,92 +452,47 @@
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>AC_td_med</t>
+          <t>AC_med</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>AC_td_lo</t>
+          <t>AC_lo</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>AC_td_hi</t>
+          <t>AC_hi</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>YLD_td_med</t>
+          <t>YLD_med</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
         <is>
-          <t>YLD_td_lo</t>
+          <t>YLD_lo</t>
         </is>
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
-          <t>YLD_td_hi</t>
+          <t>YLD_hi</t>
         </is>
       </c>
       <c r="Z1" s="1" t="inlineStr">
         <is>
-          <t>DALY_td_med</t>
+          <t>DALY_med</t>
         </is>
       </c>
       <c r="AA1" s="1" t="inlineStr">
         <is>
-          <t>DALY_td_lo</t>
+          <t>DALY_lo</t>
         </is>
       </c>
       <c r="AB1" s="1" t="inlineStr">
         <is>
-          <t>DALY_td_hi</t>
-        </is>
-      </c>
-      <c r="AC1" s="1" t="inlineStr">
-        <is>
-          <t>AC_bu_med</t>
-        </is>
-      </c>
-      <c r="AD1" s="1" t="inlineStr">
-        <is>
-          <t>AC_bu_lo</t>
-        </is>
-      </c>
-      <c r="AE1" s="1" t="inlineStr">
-        <is>
-          <t>AC_bu_hi</t>
-        </is>
-      </c>
-      <c r="AF1" s="1" t="inlineStr">
-        <is>
-          <t>YLD_bu_med</t>
-        </is>
-      </c>
-      <c r="AG1" s="1" t="inlineStr">
-        <is>
-          <t>YLD_bu_lo</t>
-        </is>
-      </c>
-      <c r="AH1" s="1" t="inlineStr">
-        <is>
-          <t>YLD_bu_hi</t>
-        </is>
-      </c>
-      <c r="AI1" s="1" t="inlineStr">
-        <is>
-          <t>DALY_bu_med</t>
-        </is>
-      </c>
-      <c r="AJ1" s="1" t="inlineStr">
-        <is>
-          <t>DALY_bu_lo</t>
-        </is>
-      </c>
-      <c r="AK1" s="1" t="inlineStr">
-        <is>
-          <t>DALY_bu_hi</t>
+          <t>DALY_hi</t>
         </is>
       </c>
     </row>
@@ -582,76 +537,49 @@
         <v>0.1719</v>
       </c>
       <c r="N2">
-        <v>0.0303147738590428</v>
+        <v>0.01205456106122915</v>
       </c>
       <c r="O2">
-        <v>0.02050873637485651</v>
+        <v>0.008060669160305015</v>
       </c>
       <c r="P2">
-        <v>0.04062063489529727</v>
+        <v>0.01606864959918909</v>
       </c>
       <c r="Q2">
-        <v>0.01186222292927166</v>
+        <v>0.004716471325574692</v>
       </c>
       <c r="R2">
-        <v>0.00668877753778795</v>
+        <v>0.002669135081370023</v>
       </c>
       <c r="S2">
-        <v>0.01845667047322525</v>
+        <v>0.007280258337832305</v>
       </c>
       <c r="T2">
-        <v>145.4464378569393</v>
+        <v>57.64719414268119</v>
       </c>
       <c r="U2">
-        <v>70.41315673181029</v>
+        <v>29.06431535475895</v>
       </c>
       <c r="V2">
-        <v>277.3782690778769</v>
+        <v>109.0972499690264</v>
       </c>
       <c r="W2">
-        <v>1.115478015053551</v>
+        <v>0.4442605848646879</v>
       </c>
       <c r="X2">
-        <v>0.4500453523181865</v>
+        <v>0.181506906688629</v>
       </c>
       <c r="Y2">
-        <v>2.622439287285581</v>
+        <v>1.026389278480296</v>
       </c>
       <c r="Z2">
-        <v>1.115478015053551</v>
+        <v>0.4442605848646879</v>
       </c>
       <c r="AA2">
-        <v>0.4500453523181865</v>
+        <v>0.181506906688629</v>
       </c>
       <c r="AB2">
-        <v>2.622439287285581</v>
-      </c>
-      <c r="AC2">
-        <v>6326.578149386855</v>
-      </c>
-      <c r="AD2">
-        <v>3567.381431709201</v>
-      </c>
-      <c r="AE2">
-        <v>9843.649779857065</v>
-      </c>
-      <c r="AF2">
-        <v>48.43278459111516</v>
-      </c>
-      <c r="AG2">
-        <v>22.09922542561096</v>
-      </c>
-      <c r="AH2">
-        <v>100.5554788563321</v>
-      </c>
-      <c r="AI2">
-        <v>48.43278459111516</v>
-      </c>
-      <c r="AJ2">
-        <v>22.09922542561096</v>
-      </c>
-      <c r="AK2">
-        <v>100.5554788563321</v>
+        <v>1.026389278480296</v>
       </c>
     </row>
   </sheetData>

</xml_diff>